<commit_message>
Drop consentGiven from SharePoint dataset columns
Collected data always has consent (enforced server-side), so a consentGiven
column would be constant and add no value. Removed it from the flat block and
the SharePoint templates/schema/docs. Consent is still recorded in
context.consentGiven for the audit trail and remains the server-side gate.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sharepoint-list-template.xlsx
+++ b/docs/sharepoint-list-template.xlsx
@@ -125,9 +125,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Submissions" displayName="Submissions" ref="A1:AS2" headerRowCount="1">
-  <autoFilter ref="A1:AS2"/>
-  <tableColumns count="45">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Submissions" displayName="Submissions" ref="A1:AR2" headerRowCount="1">
+  <autoFilter ref="A1:AR2"/>
+  <tableColumns count="44">
     <tableColumn id="1" name="submittedAt"/>
     <tableColumn id="2" name="sessionId"/>
     <tableColumn id="3" name="locale"/>
@@ -137,42 +137,41 @@
     <tableColumn id="7" name="principal"/>
     <tableColumn id="8" name="municipalitySize"/>
     <tableColumn id="9" name="privateSchoolSize"/>
-    <tableColumn id="10" name="consentGiven"/>
-    <tableColumn id="11" name="score_ANA"/>
-    <tableColumn id="12" name="avg_ANA"/>
-    <tableColumn id="13" name="priority_ANA"/>
-    <tableColumn id="14" name="score_EFF"/>
-    <tableColumn id="15" name="avg_EFF"/>
-    <tableColumn id="16" name="priority_EFF"/>
-    <tableColumn id="17" name="score_KNO"/>
-    <tableColumn id="18" name="avg_KNO"/>
-    <tableColumn id="19" name="priority_KNO"/>
-    <tableColumn id="20" name="score_SUP"/>
-    <tableColumn id="21" name="avg_SUP"/>
-    <tableColumn id="22" name="priority_SUP"/>
-    <tableColumn id="23" name="score_TEC"/>
-    <tableColumn id="24" name="avg_TEC"/>
-    <tableColumn id="25" name="priority_TEC"/>
-    <tableColumn id="26" name="q_ana_1"/>
-    <tableColumn id="27" name="q_ana_2"/>
-    <tableColumn id="28" name="q_ana_3"/>
-    <tableColumn id="29" name="q_ana_4"/>
-    <tableColumn id="30" name="q_eff_1"/>
-    <tableColumn id="31" name="q_eff_2"/>
-    <tableColumn id="32" name="q_eff_3"/>
-    <tableColumn id="33" name="q_eff_4"/>
-    <tableColumn id="34" name="q_kno_1"/>
-    <tableColumn id="35" name="q_kno_2"/>
-    <tableColumn id="36" name="q_kno_3"/>
-    <tableColumn id="37" name="q_kno_4"/>
-    <tableColumn id="38" name="q_sup_1"/>
-    <tableColumn id="39" name="q_sup_2"/>
-    <tableColumn id="40" name="q_sup_3"/>
-    <tableColumn id="41" name="q_sup_4"/>
-    <tableColumn id="42" name="q_tec_1"/>
-    <tableColumn id="43" name="q_tec_2"/>
-    <tableColumn id="44" name="q_tec_3"/>
-    <tableColumn id="45" name="q_tec_4"/>
+    <tableColumn id="10" name="score_ANA"/>
+    <tableColumn id="11" name="avg_ANA"/>
+    <tableColumn id="12" name="priority_ANA"/>
+    <tableColumn id="13" name="score_EFF"/>
+    <tableColumn id="14" name="avg_EFF"/>
+    <tableColumn id="15" name="priority_EFF"/>
+    <tableColumn id="16" name="score_KNO"/>
+    <tableColumn id="17" name="avg_KNO"/>
+    <tableColumn id="18" name="priority_KNO"/>
+    <tableColumn id="19" name="score_SUP"/>
+    <tableColumn id="20" name="avg_SUP"/>
+    <tableColumn id="21" name="priority_SUP"/>
+    <tableColumn id="22" name="score_TEC"/>
+    <tableColumn id="23" name="avg_TEC"/>
+    <tableColumn id="24" name="priority_TEC"/>
+    <tableColumn id="25" name="q_ana_1"/>
+    <tableColumn id="26" name="q_ana_2"/>
+    <tableColumn id="27" name="q_ana_3"/>
+    <tableColumn id="28" name="q_ana_4"/>
+    <tableColumn id="29" name="q_eff_1"/>
+    <tableColumn id="30" name="q_eff_2"/>
+    <tableColumn id="31" name="q_eff_3"/>
+    <tableColumn id="32" name="q_eff_4"/>
+    <tableColumn id="33" name="q_kno_1"/>
+    <tableColumn id="34" name="q_kno_2"/>
+    <tableColumn id="35" name="q_kno_3"/>
+    <tableColumn id="36" name="q_kno_4"/>
+    <tableColumn id="37" name="q_sup_1"/>
+    <tableColumn id="38" name="q_sup_2"/>
+    <tableColumn id="39" name="q_sup_3"/>
+    <tableColumn id="40" name="q_sup_4"/>
+    <tableColumn id="41" name="q_tec_1"/>
+    <tableColumn id="42" name="q_tec_2"/>
+    <tableColumn id="43" name="q_tec_3"/>
+    <tableColumn id="44" name="q_tec_4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -467,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS2"/>
+  <dimension ref="A1:AR2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -518,180 +517,175 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>consentGiven</t>
+          <t>score_ANA</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>score_ANA</t>
+          <t>avg_ANA</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>avg_ANA</t>
+          <t>priority_ANA</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>priority_ANA</t>
+          <t>score_EFF</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>score_EFF</t>
+          <t>avg_EFF</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>avg_EFF</t>
+          <t>priority_EFF</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>priority_EFF</t>
+          <t>score_KNO</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>score_KNO</t>
+          <t>avg_KNO</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>avg_KNO</t>
+          <t>priority_KNO</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>priority_KNO</t>
+          <t>score_SUP</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>score_SUP</t>
+          <t>avg_SUP</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>avg_SUP</t>
+          <t>priority_SUP</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>priority_SUP</t>
+          <t>score_TEC</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>score_TEC</t>
+          <t>avg_TEC</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>avg_TEC</t>
+          <t>priority_TEC</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
         <is>
-          <t>priority_TEC</t>
+          <t>q_ana_1</t>
         </is>
       </c>
       <c r="Z1" t="inlineStr">
         <is>
-          <t>q_ana_1</t>
+          <t>q_ana_2</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr">
         <is>
-          <t>q_ana_2</t>
+          <t>q_ana_3</t>
         </is>
       </c>
       <c r="AB1" t="inlineStr">
         <is>
-          <t>q_ana_3</t>
+          <t>q_ana_4</t>
         </is>
       </c>
       <c r="AC1" t="inlineStr">
         <is>
-          <t>q_ana_4</t>
+          <t>q_eff_1</t>
         </is>
       </c>
       <c r="AD1" t="inlineStr">
         <is>
-          <t>q_eff_1</t>
+          <t>q_eff_2</t>
         </is>
       </c>
       <c r="AE1" t="inlineStr">
         <is>
-          <t>q_eff_2</t>
+          <t>q_eff_3</t>
         </is>
       </c>
       <c r="AF1" t="inlineStr">
         <is>
-          <t>q_eff_3</t>
+          <t>q_eff_4</t>
         </is>
       </c>
       <c r="AG1" t="inlineStr">
         <is>
-          <t>q_eff_4</t>
+          <t>q_kno_1</t>
         </is>
       </c>
       <c r="AH1" t="inlineStr">
         <is>
-          <t>q_kno_1</t>
+          <t>q_kno_2</t>
         </is>
       </c>
       <c r="AI1" t="inlineStr">
         <is>
-          <t>q_kno_2</t>
+          <t>q_kno_3</t>
         </is>
       </c>
       <c r="AJ1" t="inlineStr">
         <is>
-          <t>q_kno_3</t>
+          <t>q_kno_4</t>
         </is>
       </c>
       <c r="AK1" t="inlineStr">
         <is>
-          <t>q_kno_4</t>
+          <t>q_sup_1</t>
         </is>
       </c>
       <c r="AL1" t="inlineStr">
         <is>
-          <t>q_sup_1</t>
+          <t>q_sup_2</t>
         </is>
       </c>
       <c r="AM1" t="inlineStr">
         <is>
-          <t>q_sup_2</t>
+          <t>q_sup_3</t>
         </is>
       </c>
       <c r="AN1" t="inlineStr">
         <is>
-          <t>q_sup_3</t>
+          <t>q_sup_4</t>
         </is>
       </c>
       <c r="AO1" t="inlineStr">
         <is>
-          <t>q_sup_4</t>
+          <t>q_tec_1</t>
         </is>
       </c>
       <c r="AP1" t="inlineStr">
         <is>
-          <t>q_tec_1</t>
+          <t>q_tec_2</t>
         </is>
       </c>
       <c r="AQ1" t="inlineStr">
         <is>
-          <t>q_tec_2</t>
+          <t>q_tec_3</t>
         </is>
       </c>
       <c r="AR1" t="inlineStr">
-        <is>
-          <t>q_tec_3</t>
-        </is>
-      </c>
-      <c r="AS1" t="inlineStr">
         <is>
           <t>q_tec_4</t>
         </is>
@@ -742,7 +736,6 @@
       <c r="AP2" t="inlineStr"/>
       <c r="AQ2" t="inlineStr"/>
       <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>